<commit_message>
Fix formatting of commented local WORKER_URL in config.js
</commit_message>
<xml_diff>
--- a/docs/stakeholder_matrix_ahp_CIT_260930.xlsx
+++ b/docs/stakeholder_matrix_ahp_CIT_260930.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="72" documentId="8_{FB023FA9-18DC-45B0-9F8A-DF721DFF8B70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78746A4D-EB66-4C1E-AE13-A824C9561A89}"/>
   <bookViews>
-    <workbookView xWindow="7935" yWindow="345" windowWidth="21210" windowHeight="15165" xr2:uid="{198BE654-42EA-4543-B053-C3E99F435526}"/>
+    <workbookView xWindow="-15420" yWindow="-3345" windowWidth="12150" windowHeight="20745" xr2:uid="{198BE654-42EA-4543-B053-C3E99F435526}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2893,29 +2893,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Kommentar xmlns="c5c7cef5-72b0-4130-9324-a6e7454301c2" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <TaxCatchAll xmlns="f51bab5f-0ed0-40a8-8f36-6fe936a64348" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c5c7cef5-72b0-4130-9324-a6e7454301c2">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="dokument" ma:contentTypeID="0x0101003CD881D636A33040B44CA3E28A7ACA21" ma:contentTypeVersion="19" ma:contentTypeDescription="Skapa ett nytt dokument." ma:contentTypeScope="" ma:versionID="40c4d47bd9b3326c4076fb84cac13a07">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="c5c7cef5-72b0-4130-9324-a6e7454301c2" xmlns:ns3="f51bab5f-0ed0-40a8-8f36-6fe936a64348" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e06a0d7c33d75c1cec6214f7c114a504" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3181,33 +3158,30 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{61F3BB97-E9FB-4B45-B702-18F7E1901F90}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="f51bab5f-0ed0-40a8-8f36-6fe936a64348"/>
-    <ds:schemaRef ds:uri="c5c7cef5-72b0-4130-9324-a6e7454301c2"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97DE168E-0F37-439D-90D9-E2C5C5D2DF55}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Kommentar xmlns="c5c7cef5-72b0-4130-9324-a6e7454301c2" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <TaxCatchAll xmlns="f51bab5f-0ed0-40a8-8f36-6fe936a64348" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c5c7cef5-72b0-4130-9324-a6e7454301c2">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE41993C-690A-4136-8610-4718A49FAECF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3225,4 +3199,30 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97DE168E-0F37-439D-90D9-E2C5C5D2DF55}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{61F3BB97-E9FB-4B45-B702-18F7E1901F90}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="f51bab5f-0ed0-40a8-8f36-6fe936a64348"/>
+    <ds:schemaRef ds:uri="c5c7cef5-72b0-4130-9324-a6e7454301c2"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>